<commit_message>
Update repository, scripts, etc.
</commit_message>
<xml_diff>
--- a/outputs/tablas/analisis_proceso_ot.xlsx
+++ b/outputs/tablas/analisis_proceso_ot.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="129">
   <si>
     <t xml:space="preserve">metrica</t>
   </si>
@@ -84,18 +84,18 @@
     <t xml:space="preserve">Validación de cierre</t>
   </si>
   <si>
+    <t xml:space="preserve">Clasificación de WO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WO cerrada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WO creada</t>
+  </si>
+  <si>
     <t xml:space="preserve">Asignación</t>
   </si>
   <si>
-    <t xml:space="preserve">Clasificación de WO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WO cerrada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WO creada</t>
-  </si>
-  <si>
     <t xml:space="preserve">Solicitud de información adicional</t>
   </si>
   <si>
@@ -111,6 +111,12 @@
     <t xml:space="preserve">Corrección de cierre</t>
   </si>
   <si>
+    <t xml:space="preserve">Atención al client</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reparación</t>
+  </si>
+  <si>
     <t xml:space="preserve">secuencia</t>
   </si>
   <si>
@@ -184,9 +190,6 @@
   </si>
   <si>
     <t xml:space="preserve">fuera_sla_pct</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reparación</t>
   </si>
   <si>
     <t xml:space="preserve">Mantenimiento</t>
@@ -828,28 +831,28 @@
         <v>10</v>
       </c>
       <c r="B1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="I1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="2">
@@ -912,16 +915,16 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B4" t="n">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="C4" t="n">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="D4" t="n">
-        <v>3949.25</v>
+        <v>3943.13</v>
       </c>
       <c r="E4" t="n">
         <v>3.95</v>
@@ -933,10 +936,10 @@
         <v>7.99</v>
       </c>
       <c r="H4" t="n">
-        <v>9.33</v>
+        <v>9.34</v>
       </c>
       <c r="I4" t="n">
-        <v>9.33</v>
+        <v>9.32</v>
       </c>
     </row>
     <row r="5">
@@ -1002,16 +1005,16 @@
         <v>15</v>
       </c>
       <c r="B7" t="n">
-        <v>1133</v>
+        <v>1132</v>
       </c>
       <c r="C7" t="n">
         <v>1000</v>
       </c>
       <c r="D7" t="n">
-        <v>2520.26</v>
+        <v>2518.88</v>
       </c>
       <c r="E7" t="n">
-        <v>2.22</v>
+        <v>2.23</v>
       </c>
       <c r="F7" t="n">
         <v>1.82</v>
@@ -1023,7 +1026,7 @@
         <v>5.32</v>
       </c>
       <c r="I7" t="n">
-        <v>5.96</v>
+        <v>5.95</v>
       </c>
     </row>
     <row r="8">
@@ -1057,7 +1060,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B9" t="n">
         <v>1000</v>
@@ -1086,7 +1089,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B10" t="n">
         <v>1000</v>
@@ -1231,30 +1234,88 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="B15" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="n">
+        <v>6.12</v>
+      </c>
+      <c r="E15" t="n">
+        <v>6.12</v>
+      </c>
+      <c r="F15" t="n">
+        <v>6.12</v>
+      </c>
+      <c r="G15" t="n">
+        <v>6.12</v>
+      </c>
+      <c r="H15" t="n">
+        <v>6.12</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="G16" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="H16" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" t="n">
         <v>1000</v>
       </c>
-      <c r="C15" t="n">
+      <c r="C17" t="n">
         <v>1000</v>
       </c>
-      <c r="D15" t="n">
+      <c r="D17" t="n">
         <v>0</v>
       </c>
-      <c r="E15" t="n">
+      <c r="E17" t="n">
         <v>0</v>
       </c>
-      <c r="F15" t="n">
+      <c r="F17" t="n">
         <v>0</v>
       </c>
-      <c r="G15" t="n">
+      <c r="G17" t="n">
         <v>0</v>
       </c>
-      <c r="H15" t="n">
+      <c r="H17" t="n">
         <v>0</v>
       </c>
-      <c r="I15" t="n">
+      <c r="I17" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1271,36 +1332,36 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E1" t="s">
+        <v>73</v>
+      </c>
+      <c r="F1" t="s">
+        <v>74</v>
+      </c>
+      <c r="G1" t="s">
+        <v>70</v>
+      </c>
+      <c r="H1" t="s">
         <v>82</v>
       </c>
-      <c r="B1" t="s">
-        <v>80</v>
-      </c>
-      <c r="C1" t="s">
-        <v>70</v>
-      </c>
-      <c r="D1" t="s">
-        <v>71</v>
-      </c>
-      <c r="E1" t="s">
-        <v>72</v>
-      </c>
-      <c r="F1" t="s">
-        <v>73</v>
-      </c>
-      <c r="G1" t="s">
-        <v>69</v>
-      </c>
-      <c r="H1" t="s">
-        <v>81</v>
-      </c>
       <c r="I1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B2" t="n">
         <v>5447</v>
@@ -1329,7 +1390,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B3" t="n">
         <v>2382</v>
@@ -1358,7 +1419,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B4" t="n">
         <v>1080</v>
@@ -1387,7 +1448,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B5" t="n">
         <v>1256</v>
@@ -1416,7 +1477,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B6" t="n">
         <v>111</v>
@@ -1456,33 +1517,33 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G1" t="s">
         <v>70</v>
-      </c>
-      <c r="E1" t="s">
-        <v>71</v>
-      </c>
-      <c r="F1" t="s">
-        <v>72</v>
-      </c>
-      <c r="G1" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C2" t="n">
         <v>914</v>
@@ -1502,10 +1563,10 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C3" t="n">
         <v>897</v>
@@ -1525,10 +1586,10 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B4" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C4" t="n">
         <v>947</v>
@@ -1548,10 +1609,10 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C5" t="n">
         <v>882</v>
@@ -1571,10 +1632,10 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C6" t="n">
         <v>934</v>
@@ -1594,10 +1655,10 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B7" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C7" t="n">
         <v>873</v>
@@ -1617,10 +1678,10 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B8" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C8" t="n">
         <v>392</v>
@@ -1640,10 +1701,10 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B9" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C9" t="n">
         <v>404</v>
@@ -1663,10 +1724,10 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B10" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C10" t="n">
         <v>422</v>
@@ -1686,10 +1747,10 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B11" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C11" t="n">
         <v>399</v>
@@ -1709,10 +1770,10 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B12" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C12" t="n">
         <v>371</v>
@@ -1732,10 +1793,10 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B13" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C13" t="n">
         <v>394</v>
@@ -1755,10 +1816,10 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C14" t="n">
         <v>180</v>
@@ -1778,10 +1839,10 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B15" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C15" t="n">
         <v>187</v>
@@ -1801,10 +1862,10 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B16" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C16" t="n">
         <v>192</v>
@@ -1824,10 +1885,10 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B17" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C17" t="n">
         <v>179</v>
@@ -1847,10 +1908,10 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B18" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C18" t="n">
         <v>177</v>
@@ -1870,10 +1931,10 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B19" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C19" t="n">
         <v>165</v>
@@ -1893,10 +1954,10 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B20" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C20" t="n">
         <v>211</v>
@@ -1916,10 +1977,10 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B21" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C21" t="n">
         <v>211</v>
@@ -1939,10 +2000,10 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B22" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C22" t="n">
         <v>207</v>
@@ -1962,10 +2023,10 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B23" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C23" t="n">
         <v>208</v>
@@ -1985,10 +2046,10 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B24" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C24" t="n">
         <v>218</v>
@@ -2008,10 +2069,10 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C25" t="n">
         <v>201</v>
@@ -2031,10 +2092,10 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B26" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C26" t="n">
         <v>22</v>
@@ -2054,10 +2115,10 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B27" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C27" t="n">
         <v>22</v>
@@ -2077,10 +2138,10 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B28" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C28" t="n">
         <v>17</v>
@@ -2100,10 +2161,10 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B29" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C29" t="n">
         <v>19</v>
@@ -2123,10 +2184,10 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B30" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C30" t="n">
         <v>17</v>
@@ -2146,10 +2207,10 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B31" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C31" t="n">
         <v>14</v>
@@ -2180,19 +2241,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2">
@@ -2225,21 +2286,21 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1" t="s">
         <v>51</v>
-      </c>
-      <c r="D1" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="B2" t="n">
         <v>352</v>
@@ -2253,7 +2314,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B3" t="n">
         <v>271</v>
@@ -2267,7 +2328,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B4" t="n">
         <v>124</v>
@@ -2281,7 +2342,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B5" t="n">
         <v>253</v>
@@ -2306,24 +2367,24 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1" t="s">
         <v>51</v>
       </c>
-      <c r="D1" t="s">
-        <v>49</v>
-      </c>
       <c r="E1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B2" t="n">
         <v>81</v>
@@ -2340,7 +2401,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B3" t="n">
         <v>241</v>
@@ -2357,7 +2418,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B4" t="n">
         <v>420</v>
@@ -2374,7 +2435,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B5" t="n">
         <v>258</v>
@@ -2402,21 +2463,21 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1" t="s">
         <v>51</v>
-      </c>
-      <c r="D1" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B2" t="n">
         <v>650</v>
@@ -2430,7 +2491,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B3" t="n">
         <v>350</v>
@@ -2455,16 +2516,16 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2">
@@ -2497,10 +2558,10 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="C4" t="n">
         <v>1000</v>
@@ -2511,10 +2572,10 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" t="s">
         <v>19</v>
-      </c>
-      <c r="B5" t="s">
-        <v>18</v>
       </c>
       <c r="C5" t="n">
         <v>1000</v>
@@ -2525,10 +2586,10 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C6" t="n">
         <v>1000</v>
@@ -2539,52 +2600,52 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="C7" t="n">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="D7" t="n">
-        <v>10.78</v>
+        <v>10.77</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C8" t="n">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="D8" t="n">
-        <v>10.78</v>
+        <v>10.77</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C9" t="n">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="D9" t="n">
-        <v>10.78</v>
+        <v>10.77</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" t="s">
         <v>22</v>
-      </c>
-      <c r="B10" t="s">
-        <v>15</v>
       </c>
       <c r="C10" t="n">
         <v>133</v>
@@ -2595,16 +2656,16 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" t="s">
         <v>15</v>
       </c>
-      <c r="B11" t="s">
-        <v>22</v>
-      </c>
       <c r="C11" t="n">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D11" t="n">
-        <v>1.43</v>
+        <v>1.42</v>
       </c>
     </row>
     <row r="12">
@@ -2717,6 +2778,62 @@
       </c>
       <c r="D19" t="n">
         <v>0.86</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" t="s">
+        <v>28</v>
+      </c>
+      <c r="C21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>28</v>
+      </c>
+      <c r="B22" t="s">
+        <v>13</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>27</v>
+      </c>
+      <c r="C23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0.01</v>
       </c>
     </row>
   </sheetData>
@@ -2768,10 +2885,10 @@
         <v>15</v>
       </c>
       <c r="B4" t="n">
-        <v>1133</v>
+        <v>1132</v>
       </c>
       <c r="C4" t="n">
-        <v>11.03</v>
+        <v>11.02</v>
       </c>
     </row>
     <row r="5">
@@ -2834,10 +2951,10 @@
         <v>21</v>
       </c>
       <c r="B10" t="n">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="C10" t="n">
-        <v>9.73</v>
+        <v>9.72</v>
       </c>
     </row>
     <row r="11">
@@ -2893,6 +3010,28 @@
       </c>
       <c r="C15" t="n">
         <v>0.78</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>28</v>
+      </c>
+      <c r="B17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.01</v>
       </c>
     </row>
   </sheetData>
@@ -2908,24 +3047,24 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B1" t="s">
         <v>11</v>
       </c>
       <c r="C1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B2" t="n">
         <v>9</v>
@@ -2942,7 +3081,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B3" t="n">
         <v>11</v>
@@ -2951,15 +3090,15 @@
         <v>2</v>
       </c>
       <c r="D3" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E3" t="n">
-        <v>6</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B4" t="n">
         <v>11</v>
@@ -2976,7 +3115,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B5" t="n">
         <v>13</v>
@@ -2993,7 +3132,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B6" t="n">
         <v>11</v>
@@ -3010,7 +3149,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B7" t="n">
         <v>11</v>
@@ -3027,7 +3166,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B8" t="n">
         <v>15</v>
@@ -3044,7 +3183,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B9" t="n">
         <v>13</v>
@@ -3061,7 +3200,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B10" t="n">
         <v>15</v>
@@ -3078,7 +3217,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B11" t="n">
         <v>13</v>
@@ -3106,28 +3245,28 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="2">
@@ -3169,27 +3308,27 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E1" t="s">
         <v>48</v>
       </c>
-      <c r="B1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D1" t="s">
-        <v>50</v>
-      </c>
-      <c r="E1" t="s">
-        <v>46</v>
-      </c>
       <c r="F1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="B2" t="n">
         <v>352</v>
@@ -3209,7 +3348,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B3" t="n">
         <v>271</v>
@@ -3229,7 +3368,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B4" t="n">
         <v>124</v>
@@ -3249,7 +3388,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B5" t="n">
         <v>253</v>
@@ -3280,27 +3419,27 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B2" t="n">
         <v>81</v>
@@ -3320,7 +3459,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B3" t="n">
         <v>241</v>
@@ -3340,7 +3479,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B4" t="n">
         <v>420</v>
@@ -3360,7 +3499,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B5" t="n">
         <v>258</v>
@@ -3391,30 +3530,30 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B2" t="n">
         <v>650</v>
@@ -3437,7 +3576,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B3" t="n">
         <v>167</v>
@@ -3460,7 +3599,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B4" t="n">
         <v>183</v>
@@ -3494,27 +3633,27 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B2" t="n">
         <v>650</v>
@@ -3534,7 +3673,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B3" t="n">
         <v>350</v>
@@ -3565,30 +3704,30 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B2" t="n">
         <v>444</v>
@@ -3611,7 +3750,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B3" t="n">
         <v>246</v>
@@ -3634,7 +3773,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B4" t="n">
         <v>160</v>
@@ -3657,7 +3796,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B5" t="n">
         <v>266</v>
@@ -3680,7 +3819,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B6" t="n">
         <v>160</v>

</xml_diff>

<commit_message>
Update repository, scripts, plots, etc.
</commit_message>
<xml_diff>
--- a/outputs/tablas/analisis_proceso_ot.xlsx
+++ b/outputs/tablas/analisis_proceso_ot.xlsx
@@ -111,85 +111,85 @@
     <t xml:space="preserve">Corrección de cierre</t>
   </si>
   <si>
-    <t xml:space="preserve">Atención al client</t>
+    <t xml:space="preserve">Instalació</t>
+  </si>
+  <si>
+    <t xml:space="preserve">secuencia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cantidad_loops</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cantidad_ot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">porcentaje_ot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WO creada -&gt; Validación inicial -&gt; Clasificación de WO -&gt; Asignación -&gt; Agenda coordinada -&gt; Trabajo iniciado -&gt; Trabajo finalizado -&gt; Validación de cierre -&gt; WO cerrada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WO creada -&gt; Validación inicial -&gt; Solicitud de información adicional -&gt; Validación inicial -&gt; Clasificación de WO -&gt; Asignación -&gt; Agenda coordinada -&gt; Trabajo iniciado -&gt; Trabajo finalizado -&gt; Validación de cierre -&gt; WO cerrada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WO creada -&gt; Validación inicial -&gt; Clasificación de WO -&gt; Asignación -&gt; Agenda coordinada -&gt; Contacto con cliente para reagendar -&gt; Agenda coordinada -&gt; Trabajo iniciado -&gt; Trabajo finalizado -&gt; Validación de cierre -&gt; WO cerrada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WO creada -&gt; Validación inicial -&gt; Clasificación de WO -&gt; Asignación -&gt; Agenda coordinada -&gt; Trabajo iniciado -&gt; Solicitud de material -&gt; Material preparado -&gt; Agenda coordinada -&gt; Trabajo iniciado -&gt; Trabajo finalizado -&gt; Validación de cierre -&gt; WO cerrada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WO creada -&gt; Validación inicial -&gt; Clasificación de WO -&gt; Asignación -&gt; Agenda coordinada -&gt; Trabajo iniciado -&gt; Trabajo finalizado -&gt; Trabajo iniciado -&gt; Trabajo finalizado -&gt; Validación de cierre -&gt; WO cerrada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WO creada -&gt; Validación inicial -&gt; Clasificación de WO -&gt; Asignación -&gt; Agenda coordinada -&gt; Trabajo iniciado -&gt; Trabajo finalizado -&gt; Validación de cierre -&gt; Corrección de cierre -&gt; Validación de cierre -&gt; WO cerrada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WO creada -&gt; Validación inicial -&gt; Clasificación de WO -&gt; Asignación -&gt; Agenda coordinada -&gt; Contacto con cliente para reagendar -&gt; Agenda coordinada -&gt; Trabajo iniciado -&gt; Solicitud de material -&gt; Material preparado -&gt; Agenda coordinada -&gt; Trabajo iniciado -&gt; Trabajo finalizado -&gt; Validación de cierre -&gt; WO cerrada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WO creada -&gt; Validación inicial -&gt; Solicitud de información adicional -&gt; Validación inicial -&gt; Clasificación de WO -&gt; Asignación -&gt; Agenda coordinada -&gt; Contacto con cliente para reagendar -&gt; Agenda coordinada -&gt; Trabajo iniciado -&gt; Trabajo finalizado -&gt; Validación de cierre -&gt; WO cerrada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WO creada -&gt; Validación inicial -&gt; Solicitud de información adicional -&gt; Validación inicial -&gt; Clasificación de WO -&gt; Asignación -&gt; Agenda coordinada -&gt; Trabajo iniciado -&gt; Solicitud de material -&gt; Material preparado -&gt; Agenda coordinada -&gt; Trabajo iniciado -&gt; Trabajo finalizado -&gt; Validación de cierre -&gt; WO cerrada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WO creada -&gt; Validación inicial -&gt; Solicitud de información adicional -&gt; Validación inicial -&gt; Clasificación de WO -&gt; Asignación -&gt; Agenda coordinada -&gt; Trabajo iniciado -&gt; Trabajo finalizado -&gt; Validación de cierre -&gt; Corrección de cierre -&gt; Validación de cierre -&gt; WO cerrada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">promedio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mediana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">p25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">p75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">p90</t>
+  </si>
+  <si>
+    <t xml:space="preserve">p95</t>
+  </si>
+  <si>
+    <t xml:space="preserve">maximo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tipo_ot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lead_time_promedio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lead_time_mediano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fuera_sla_pct</t>
   </si>
   <si>
     <t xml:space="preserve">Reparación</t>
-  </si>
-  <si>
-    <t xml:space="preserve">secuencia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cantidad_loops</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cantidad_ot</t>
-  </si>
-  <si>
-    <t xml:space="preserve">porcentaje_ot</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WO creada -&gt; Validación inicial -&gt; Clasificación de WO -&gt; Asignación -&gt; Agenda coordinada -&gt; Trabajo iniciado -&gt; Trabajo finalizado -&gt; Validación de cierre -&gt; WO cerrada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WO creada -&gt; Validación inicial -&gt; Solicitud de información adicional -&gt; Validación inicial -&gt; Clasificación de WO -&gt; Asignación -&gt; Agenda coordinada -&gt; Trabajo iniciado -&gt; Trabajo finalizado -&gt; Validación de cierre -&gt; WO cerrada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WO creada -&gt; Validación inicial -&gt; Clasificación de WO -&gt; Asignación -&gt; Agenda coordinada -&gt; Contacto con cliente para reagendar -&gt; Agenda coordinada -&gt; Trabajo iniciado -&gt; Trabajo finalizado -&gt; Validación de cierre -&gt; WO cerrada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WO creada -&gt; Validación inicial -&gt; Clasificación de WO -&gt; Asignación -&gt; Agenda coordinada -&gt; Trabajo iniciado -&gt; Solicitud de material -&gt; Material preparado -&gt; Agenda coordinada -&gt; Trabajo iniciado -&gt; Trabajo finalizado -&gt; Validación de cierre -&gt; WO cerrada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WO creada -&gt; Validación inicial -&gt; Clasificación de WO -&gt; Asignación -&gt; Agenda coordinada -&gt; Trabajo iniciado -&gt; Trabajo finalizado -&gt; Trabajo iniciado -&gt; Trabajo finalizado -&gt; Validación de cierre -&gt; WO cerrada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WO creada -&gt; Validación inicial -&gt; Clasificación de WO -&gt; Asignación -&gt; Agenda coordinada -&gt; Trabajo iniciado -&gt; Trabajo finalizado -&gt; Validación de cierre -&gt; Corrección de cierre -&gt; Validación de cierre -&gt; WO cerrada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WO creada -&gt; Validación inicial -&gt; Clasificación de WO -&gt; Asignación -&gt; Agenda coordinada -&gt; Contacto con cliente para reagendar -&gt; Agenda coordinada -&gt; Trabajo iniciado -&gt; Solicitud de material -&gt; Material preparado -&gt; Agenda coordinada -&gt; Trabajo iniciado -&gt; Trabajo finalizado -&gt; Validación de cierre -&gt; WO cerrada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WO creada -&gt; Validación inicial -&gt; Solicitud de información adicional -&gt; Validación inicial -&gt; Clasificación de WO -&gt; Asignación -&gt; Agenda coordinada -&gt; Contacto con cliente para reagendar -&gt; Agenda coordinada -&gt; Trabajo iniciado -&gt; Trabajo finalizado -&gt; Validación de cierre -&gt; WO cerrada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WO creada -&gt; Validación inicial -&gt; Solicitud de información adicional -&gt; Validación inicial -&gt; Clasificación de WO -&gt; Asignación -&gt; Agenda coordinada -&gt; Trabajo iniciado -&gt; Solicitud de material -&gt; Material preparado -&gt; Agenda coordinada -&gt; Trabajo iniciado -&gt; Trabajo finalizado -&gt; Validación de cierre -&gt; WO cerrada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WO creada -&gt; Validación inicial -&gt; Solicitud de información adicional -&gt; Validación inicial -&gt; Clasificación de WO -&gt; Asignación -&gt; Agenda coordinada -&gt; Trabajo iniciado -&gt; Trabajo finalizado -&gt; Validación de cierre -&gt; Corrección de cierre -&gt; Validación de cierre -&gt; WO cerrada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">promedio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mediana</t>
-  </si>
-  <si>
-    <t xml:space="preserve">p25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">p75</t>
-  </si>
-  <si>
-    <t xml:space="preserve">p90</t>
-  </si>
-  <si>
-    <t xml:space="preserve">p95</t>
-  </si>
-  <si>
-    <t xml:space="preserve">maximo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tipo_ot</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lead_time_promedio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lead_time_mediano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fuera_sla_pct</t>
   </si>
   <si>
     <t xml:space="preserve">Mantenimiento</t>
@@ -846,10 +846,10 @@
         <v>74</v>
       </c>
       <c r="G1" t="s">
+        <v>46</v>
+      </c>
+      <c r="H1" t="s">
         <v>47</v>
-      </c>
-      <c r="H1" t="s">
-        <v>48</v>
       </c>
       <c r="I1" t="s">
         <v>82</v>
@@ -924,22 +924,22 @@
         <v>999</v>
       </c>
       <c r="D4" t="n">
-        <v>3943.13</v>
+        <v>3940.12</v>
       </c>
       <c r="E4" t="n">
-        <v>3.95</v>
+        <v>3.94</v>
       </c>
       <c r="F4" t="n">
         <v>3.22</v>
       </c>
       <c r="G4" t="n">
-        <v>7.99</v>
+        <v>7.98</v>
       </c>
       <c r="H4" t="n">
         <v>9.34</v>
       </c>
       <c r="I4" t="n">
-        <v>9.32</v>
+        <v>9.31</v>
       </c>
     </row>
     <row r="5">
@@ -1005,16 +1005,16 @@
         <v>15</v>
       </c>
       <c r="B7" t="n">
-        <v>1132</v>
+        <v>1133</v>
       </c>
       <c r="C7" t="n">
         <v>1000</v>
       </c>
       <c r="D7" t="n">
-        <v>2518.88</v>
+        <v>2520.26</v>
       </c>
       <c r="E7" t="n">
-        <v>2.23</v>
+        <v>2.22</v>
       </c>
       <c r="F7" t="n">
         <v>1.82</v>
@@ -1026,7 +1026,7 @@
         <v>5.32</v>
       </c>
       <c r="I7" t="n">
-        <v>5.95</v>
+        <v>5.96</v>
       </c>
     </row>
     <row r="8">
@@ -1234,7 +1234,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B15" t="n">
         <v>1</v>
@@ -1243,79 +1243,50 @@
         <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>6.12</v>
+        <v>9.13</v>
       </c>
       <c r="E15" t="n">
-        <v>6.12</v>
+        <v>9.13</v>
       </c>
       <c r="F15" t="n">
-        <v>6.12</v>
+        <v>9.13</v>
       </c>
       <c r="G15" t="n">
-        <v>6.12</v>
+        <v>9.13</v>
       </c>
       <c r="H15" t="n">
-        <v>6.12</v>
+        <v>9.13</v>
       </c>
       <c r="I15" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="D16" t="n">
-        <v>1.38</v>
+        <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>1.38</v>
+        <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>1.38</v>
+        <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>1.38</v>
+        <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>1.38</v>
+        <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="s">
-        <v>20</v>
-      </c>
-      <c r="B17" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C17" t="n">
-        <v>1000</v>
-      </c>
-      <c r="D17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2241,13 +2212,13 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
         <v>121</v>
       </c>
       <c r="C1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D1" t="s">
         <v>122</v>
@@ -2286,21 +2257,21 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D1" t="s">
         <v>50</v>
-      </c>
-      <c r="B1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1" t="s">
-        <v>53</v>
-      </c>
-      <c r="D1" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>28</v>
+        <v>53</v>
       </c>
       <c r="B2" t="n">
         <v>352</v>
@@ -2370,13 +2341,13 @@
         <v>57</v>
       </c>
       <c r="B1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E1" t="s">
         <v>124</v>
@@ -2466,13 +2437,13 @@
         <v>66</v>
       </c>
       <c r="B1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2">
@@ -2586,10 +2557,10 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C6" t="n">
         <v>1000</v>
@@ -2600,24 +2571,24 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C7" t="n">
-        <v>999</v>
+        <v>1000</v>
       </c>
       <c r="D7" t="n">
-        <v>10.77</v>
+        <v>10.78</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="C8" t="n">
         <v>999</v>
@@ -2628,10 +2599,10 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B9" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C9" t="n">
         <v>999</v>
@@ -2642,10 +2613,10 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" t="s">
         <v>15</v>
-      </c>
-      <c r="B10" t="s">
-        <v>22</v>
       </c>
       <c r="C10" t="n">
         <v>133</v>
@@ -2656,16 +2627,16 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" t="s">
         <v>22</v>
       </c>
-      <c r="B11" t="s">
-        <v>15</v>
-      </c>
       <c r="C11" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D11" t="n">
-        <v>1.42</v>
+        <v>1.43</v>
       </c>
     </row>
     <row r="12">
@@ -2782,10 +2753,10 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
+        <v>18</v>
+      </c>
+      <c r="B20" t="s">
         <v>27</v>
-      </c>
-      <c r="B20" t="s">
-        <v>18</v>
       </c>
       <c r="C20" t="n">
         <v>1</v>
@@ -2796,43 +2767,15 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="B21" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="C21" t="n">
         <v>1</v>
       </c>
       <c r="D21" t="n">
-        <v>0.01</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="s">
-        <v>28</v>
-      </c>
-      <c r="B22" t="s">
-        <v>13</v>
-      </c>
-      <c r="C22" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" t="n">
-        <v>0.01</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="s">
-        <v>22</v>
-      </c>
-      <c r="B23" t="s">
-        <v>27</v>
-      </c>
-      <c r="C23" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" t="n">
         <v>0.01</v>
       </c>
     </row>
@@ -2885,10 +2828,10 @@
         <v>15</v>
       </c>
       <c r="B4" t="n">
-        <v>1132</v>
+        <v>1133</v>
       </c>
       <c r="C4" t="n">
-        <v>11.02</v>
+        <v>11.03</v>
       </c>
     </row>
     <row r="5">
@@ -3020,17 +2963,6 @@
         <v>1</v>
       </c>
       <c r="C16" t="n">
-        <v>0.01</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="s">
-        <v>28</v>
-      </c>
-      <c r="B17" t="n">
-        <v>1</v>
-      </c>
-      <c r="C17" t="n">
         <v>0.01</v>
       </c>
     </row>
@@ -3047,24 +2979,24 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B1" t="s">
         <v>11</v>
       </c>
       <c r="C1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1" t="s">
         <v>30</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>31</v>
-      </c>
-      <c r="E1" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B2" t="n">
         <v>9</v>
@@ -3073,15 +3005,15 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="E2" t="n">
-        <v>65</v>
+        <v>64.9</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B3" t="n">
         <v>11</v>
@@ -3090,15 +3022,15 @@
         <v>2</v>
       </c>
       <c r="D3" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E3" t="n">
-        <v>5.9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B4" t="n">
         <v>11</v>
@@ -3115,7 +3047,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B5" t="n">
         <v>13</v>
@@ -3132,7 +3064,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B6" t="n">
         <v>11</v>
@@ -3149,7 +3081,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B7" t="n">
         <v>11</v>
@@ -3166,7 +3098,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B8" t="n">
         <v>15</v>
@@ -3183,7 +3115,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B9" t="n">
         <v>13</v>
@@ -3200,7 +3132,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B10" t="n">
         <v>15</v>
@@ -3217,7 +3149,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B11" t="n">
         <v>13</v>
@@ -3245,28 +3177,28 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1" t="s">
         <v>43</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>44</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>45</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>46</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>47</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>48</v>
-      </c>
-      <c r="H1" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="2">
@@ -3308,27 +3240,27 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" t="s">
         <v>50</v>
       </c>
-      <c r="B1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>51</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F1" t="s">
         <v>52</v>
-      </c>
-      <c r="E1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F1" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>28</v>
+        <v>53</v>
       </c>
       <c r="B2" t="n">
         <v>352</v>
@@ -3422,19 +3354,19 @@
         <v>57</v>
       </c>
       <c r="B1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" t="s">
         <v>51</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F1" t="s">
         <v>52</v>
-      </c>
-      <c r="E1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F1" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="2">
@@ -3533,22 +3465,22 @@
         <v>62</v>
       </c>
       <c r="B1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" t="s">
         <v>31</v>
       </c>
-      <c r="C1" t="s">
-        <v>32</v>
-      </c>
       <c r="D1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1" t="s">
         <v>51</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
+        <v>47</v>
+      </c>
+      <c r="G1" t="s">
         <v>52</v>
-      </c>
-      <c r="F1" t="s">
-        <v>48</v>
-      </c>
-      <c r="G1" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="2">
@@ -3636,19 +3568,19 @@
         <v>66</v>
       </c>
       <c r="B1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" t="s">
         <v>31</v>
       </c>
-      <c r="C1" t="s">
-        <v>32</v>
-      </c>
       <c r="D1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1" t="s">
         <v>51</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>52</v>
-      </c>
-      <c r="F1" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="2">

</xml_diff>